<commit_message>
data: screener run 2026-08-10
</commit_message>
<xml_diff>
--- a/factor_output.xlsx
+++ b/factor_output.xlsx
@@ -47167,7 +47167,7 @@
     <row r="2">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Generated: 2026-08-07</t>
+          <t>Generated: 2026-08-10</t>
         </is>
       </c>
     </row>
@@ -48465,7 +48465,7 @@
     <row r="2">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Generated: 2026-08-07</t>
+          <t>Generated: 2026-08-10</t>
         </is>
       </c>
     </row>
@@ -49838,7 +49838,7 @@
       </c>
       <c r="B54" s="27" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-10</t>
         </is>
       </c>
     </row>

</xml_diff>